<commit_message>
Daily EOD data and reports for 2026-09-10
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260910.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260910.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.882</v>
+        <v>1.88</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.008</v>
+        <v>-0.01</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.42%</t>
+          <t>-0.53%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>288286.64</v>
+        <v>287980.28</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-1225.45</v>
+        <v>-1531.81</v>
       </c>
     </row>
     <row r="5">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>62.475</v>
+        <v>62.43</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-2.105</v>
+        <v>-2.15</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-3.26%</t>
+          <t>-3.33%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>499800</v>
+        <v>499440</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-16840</v>
+        <v>-17200</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>152.3</v>
+        <v>152.2</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.95</v>
+        <v>-3.05</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.90%</t>
+          <t>-1.96%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>168.48</v>
+        <v>168.315</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-2.73</v>
+        <v>-2.895</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-1.59%</t>
+          <t>-1.69%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>673920</v>
+        <v>673260</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-10920</v>
+        <v>-11580</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.70%</t>
+          <t>7.41%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5600</v>
+        <v>5800</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.095</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.095</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-570</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.9</v>
+        <v>33.88</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.49</v>
+        <v>-0.51</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.42%</t>
+          <t>-1.48%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.89</v>
+        <v>32.885</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.25</v>
+        <v>-0.255</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42362.32</v>
+        <v>42355.88</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-322</v>
+        <v>-328.44</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1691489.41</v>
+        <v>1690926.61</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-33315.71</v>
+        <v>-33878.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>